<commit_message>
depths of duplicated stations
</commit_message>
<xml_diff>
--- a/data/su_si_duplicates_depths.xlsx
+++ b/data/su_si_duplicates_depths.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\fish_biodiversity\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F8D0A858-35F6-4108-ABB5-65B3FCA69154}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{357D8D24-0EDC-4EA2-A09D-AC411CEE4740}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-19310" yWindow="4200" windowWidth="19420" windowHeight="11020" xr2:uid="{BDA2F0B1-24DB-4159-8969-BC3C7300995E}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="38">
   <si>
     <t>Match_ID</t>
   </si>
@@ -117,13 +117,46 @@
   </si>
   <si>
     <t>si_depth</t>
+  </si>
+  <si>
+    <t>sea</t>
+  </si>
+  <si>
+    <t>bohol</t>
+  </si>
+  <si>
+    <t>sulu</t>
+  </si>
+  <si>
+    <t>lagoon</t>
+  </si>
+  <si>
+    <t>mangrove</t>
+  </si>
+  <si>
+    <t>reef</t>
+  </si>
+  <si>
+    <t>habitat</t>
+  </si>
+  <si>
+    <t>retain</t>
+  </si>
+  <si>
+    <t>filter</t>
+  </si>
+  <si>
+    <t>depth_median_sea</t>
+  </si>
+  <si>
+    <t>depth_avg_sea</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -139,13 +172,25 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -157,14 +202,21 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1"/>
+    <xf numFmtId="1" fontId="2" fillId="2" borderId="0" xfId="1" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="2" fillId="2" borderId="0" xfId="1" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Bad" xfId="1" builtinId="27"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -497,13 +549,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7B2447B-3F98-424D-A0F1-71364B25FA83}">
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="1" max="1" width="16.1015625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.15625" customWidth="1"/>
+    <col min="2" max="2" width="7.83984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.26171875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.83984375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.5234375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -513,42 +569,102 @@
       <c r="C1" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="D1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" t="s">
+        <v>33</v>
+      </c>
+      <c r="F1" t="s">
+        <v>34</v>
+      </c>
+      <c r="G1" t="s">
+        <v>36</v>
+      </c>
+      <c r="H1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" t="s">
         <v>1</v>
       </c>
-      <c r="B2">
+      <c r="B2" s="1">
         <v>30</v>
       </c>
-      <c r="C2">
+      <c r="C2" s="1">
         <v>30.5</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="D2" t="s">
+        <v>28</v>
+      </c>
+      <c r="E2" t="s">
+        <v>32</v>
+      </c>
+      <c r="F2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G2" s="5">
+        <v>6.1</v>
+      </c>
+      <c r="H2" s="5">
+        <v>10.029999999999999</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" t="s">
         <v>2</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="1">
         <v>10.7</v>
       </c>
-      <c r="C3">
+      <c r="C3" s="1">
         <v>10.7</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="D3" t="s">
+        <v>28</v>
+      </c>
+      <c r="E3" t="s">
+        <v>32</v>
+      </c>
+      <c r="F3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G3" s="5">
+        <v>6.1</v>
+      </c>
+      <c r="H3" s="5">
+        <v>10.029999999999999</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" t="s">
         <v>3</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="1">
         <v>6</v>
       </c>
-      <c r="C4">
-        <v>6.1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A5" s="1" t="s">
+      <c r="C4" s="1">
+        <v>6.1</v>
+      </c>
+      <c r="D4" t="s">
+        <v>28</v>
+      </c>
+      <c r="E4" t="s">
+        <v>32</v>
+      </c>
+      <c r="F4" t="s">
+        <v>34</v>
+      </c>
+      <c r="G4" s="5">
+        <v>6.1</v>
+      </c>
+      <c r="H4" s="5">
+        <v>10.029999999999999</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A5" t="s">
         <v>4</v>
       </c>
       <c r="B5" s="1">
@@ -557,20 +673,50 @@
       <c r="C5" s="1">
         <v>3</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="D5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E5" t="s">
+        <v>32</v>
+      </c>
+      <c r="F5" t="s">
+        <v>34</v>
+      </c>
+      <c r="G5" s="5">
+        <v>6.1</v>
+      </c>
+      <c r="H5" s="5">
+        <v>10.029999999999999</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" t="s">
         <v>5</v>
       </c>
-      <c r="B6">
+      <c r="B6" s="1">
         <v>2.5</v>
       </c>
-      <c r="C6">
+      <c r="C6" s="1">
         <v>2</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A7" s="1" t="s">
+      <c r="D6" t="s">
+        <v>28</v>
+      </c>
+      <c r="E6" t="s">
+        <v>32</v>
+      </c>
+      <c r="F6" t="s">
+        <v>34</v>
+      </c>
+      <c r="G6" s="5">
+        <v>6.1</v>
+      </c>
+      <c r="H6" s="5">
+        <v>10.029999999999999</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A7" t="s">
         <v>6</v>
       </c>
       <c r="B7" s="1">
@@ -579,186 +725,497 @@
       <c r="C7" s="1">
         <v>2</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="D7" t="s">
+        <v>28</v>
+      </c>
+      <c r="E7" t="s">
+        <v>32</v>
+      </c>
+      <c r="F7" t="s">
+        <v>34</v>
+      </c>
+      <c r="G7" s="5">
+        <v>6.1</v>
+      </c>
+      <c r="H7" s="5">
+        <v>10.029999999999999</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" t="s">
         <v>7</v>
       </c>
-      <c r="B8">
+      <c r="B8" s="1">
         <v>9.1</v>
       </c>
-      <c r="C8">
+      <c r="C8" s="1">
         <v>9.1</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="D8" t="s">
+        <v>28</v>
+      </c>
+      <c r="E8" t="s">
+        <v>32</v>
+      </c>
+      <c r="F8" t="s">
+        <v>34</v>
+      </c>
+      <c r="G8" s="5">
+        <v>6.1</v>
+      </c>
+      <c r="H8" s="5">
+        <v>10.029999999999999</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" t="s">
         <v>8</v>
       </c>
-      <c r="B9">
+      <c r="B9" s="1">
         <v>3</v>
       </c>
-      <c r="C9">
+      <c r="C9" s="1">
         <v>3</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="D9" t="s">
+        <v>28</v>
+      </c>
+      <c r="E9" t="s">
+        <v>32</v>
+      </c>
+      <c r="F9" t="s">
+        <v>34</v>
+      </c>
+      <c r="G9" s="5">
+        <v>6.1</v>
+      </c>
+      <c r="H9" s="5">
+        <v>10.029999999999999</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" t="s">
         <v>9</v>
       </c>
-      <c r="B10">
+      <c r="B10" s="1">
         <v>4.5999999999999996</v>
       </c>
-      <c r="C10">
+      <c r="C10" s="1">
         <v>4.5999999999999996</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A11" t="s">
+      <c r="D10" t="s">
+        <v>29</v>
+      </c>
+      <c r="E10" t="s">
+        <v>32</v>
+      </c>
+      <c r="F10" t="s">
+        <v>34</v>
+      </c>
+      <c r="G10" s="5">
+        <v>9.15</v>
+      </c>
+      <c r="H10" s="5">
+        <v>9.59</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A11" s="3" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="B11" s="4">
+        <v>1</v>
+      </c>
+      <c r="C11" s="4">
+        <v>1</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="G11" s="6">
+        <v>9.15</v>
+      </c>
+      <c r="H11" s="6">
+        <v>9.59</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" t="s">
         <v>11</v>
       </c>
-      <c r="B12">
+      <c r="B12" s="1">
         <v>13.64</v>
       </c>
-      <c r="C12">
+      <c r="C12" s="1">
         <v>13.7</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="D12" t="s">
+        <v>29</v>
+      </c>
+      <c r="E12" t="s">
+        <v>32</v>
+      </c>
+      <c r="F12" t="s">
+        <v>34</v>
+      </c>
+      <c r="G12" s="5">
+        <v>9.15</v>
+      </c>
+      <c r="H12" s="5">
+        <v>9.59</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" t="s">
         <v>12</v>
       </c>
-      <c r="B13">
+      <c r="B13" s="1">
         <v>21.21</v>
       </c>
-      <c r="C13">
+      <c r="C13" s="1">
         <v>21.3</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="D13" t="s">
+        <v>29</v>
+      </c>
+      <c r="E13" t="s">
+        <v>32</v>
+      </c>
+      <c r="F13" t="s">
+        <v>34</v>
+      </c>
+      <c r="G13" s="5">
+        <v>9.15</v>
+      </c>
+      <c r="H13" s="5">
+        <v>9.59</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" t="s">
         <v>13</v>
       </c>
-      <c r="B14">
+      <c r="B14" s="1">
         <v>17.27</v>
       </c>
-      <c r="C14">
+      <c r="C14" s="1">
         <v>17.399999999999999</v>
       </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="D14" t="s">
+        <v>29</v>
+      </c>
+      <c r="E14" t="s">
+        <v>32</v>
+      </c>
+      <c r="F14" t="s">
+        <v>34</v>
+      </c>
+      <c r="G14" s="5">
+        <v>9.15</v>
+      </c>
+      <c r="H14" s="5">
+        <v>9.59</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" t="s">
         <v>14</v>
       </c>
-      <c r="B15">
+      <c r="B15" s="1">
         <v>13.64</v>
       </c>
-      <c r="C15">
+      <c r="C15" s="1">
         <v>13.7</v>
       </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="D15" t="s">
+        <v>29</v>
+      </c>
+      <c r="E15" t="s">
+        <v>32</v>
+      </c>
+      <c r="F15" t="s">
+        <v>34</v>
+      </c>
+      <c r="G15" s="5">
+        <v>9.15</v>
+      </c>
+      <c r="H15" s="5">
+        <v>9.59</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" t="s">
         <v>15</v>
       </c>
-      <c r="B16">
+      <c r="B16" s="1">
         <v>3.03</v>
       </c>
-      <c r="C16">
+      <c r="C16" s="1">
         <v>3</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="D16" t="s">
+        <v>29</v>
+      </c>
+      <c r="E16" t="s">
+        <v>32</v>
+      </c>
+      <c r="F16" t="s">
+        <v>34</v>
+      </c>
+      <c r="G16" s="5">
+        <v>9.15</v>
+      </c>
+      <c r="H16" s="5">
+        <v>9.59</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" t="s">
         <v>16</v>
       </c>
-      <c r="B17">
+      <c r="B17" s="1">
         <v>2.42</v>
       </c>
-      <c r="C17">
+      <c r="C17" s="1">
         <v>2</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A18" t="s">
+      <c r="D17" t="s">
+        <v>29</v>
+      </c>
+      <c r="E17" t="s">
+        <v>32</v>
+      </c>
+      <c r="F17" t="s">
+        <v>34</v>
+      </c>
+      <c r="G17" s="5">
+        <v>9.15</v>
+      </c>
+      <c r="H17" s="5">
+        <v>9.59</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A18" s="3" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="B18" s="4">
+        <v>1</v>
+      </c>
+      <c r="C18" s="4">
+        <v>1</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="G18" s="6">
+        <v>9.15</v>
+      </c>
+      <c r="H18" s="6">
+        <v>9.59</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" t="s">
         <v>18</v>
       </c>
-      <c r="B19">
+      <c r="B19" s="1">
         <v>1.21</v>
       </c>
-      <c r="C19">
+      <c r="C19" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="D19" t="s">
+        <v>29</v>
+      </c>
+      <c r="E19" t="s">
+        <v>32</v>
+      </c>
+      <c r="F19" t="s">
+        <v>34</v>
+      </c>
+      <c r="G19" s="5">
+        <v>9.15</v>
+      </c>
+      <c r="H19" s="5">
+        <v>9.59</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" t="s">
         <v>19</v>
       </c>
-      <c r="B20">
+      <c r="B20" s="1">
         <v>18.3</v>
       </c>
-      <c r="C20">
+      <c r="C20" s="1">
         <v>18.3</v>
       </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="D20" t="s">
+        <v>28</v>
+      </c>
+      <c r="E20" t="s">
+        <v>32</v>
+      </c>
+      <c r="F20" t="s">
+        <v>34</v>
+      </c>
+      <c r="G20" s="5">
+        <v>6.1</v>
+      </c>
+      <c r="H20" s="5">
+        <v>10.029999999999999</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A21" t="s">
         <v>20</v>
       </c>
-      <c r="B21">
+      <c r="B21" s="1">
         <v>12</v>
       </c>
-      <c r="C21">
+      <c r="C21" s="1">
         <v>12.2</v>
       </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A22" t="s">
+      <c r="D21" t="s">
+        <v>28</v>
+      </c>
+      <c r="E21" t="s">
+        <v>32</v>
+      </c>
+      <c r="F21" t="s">
+        <v>34</v>
+      </c>
+      <c r="G21" s="5">
+        <v>6.1</v>
+      </c>
+      <c r="H21" s="5">
+        <v>10.029999999999999</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A22" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="B22" s="4">
+        <v>2</v>
+      </c>
+      <c r="C22" s="4">
+        <v>2</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="F22" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="G22" s="6">
+        <v>6.1</v>
+      </c>
+      <c r="H22" s="6">
+        <v>10.029999999999999</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" t="s">
         <v>22</v>
       </c>
-      <c r="B23" s="1">
+      <c r="B23" s="2">
         <v>2</v>
       </c>
-      <c r="C23" s="1">
+      <c r="C23" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="D23" t="s">
+        <v>28</v>
+      </c>
+      <c r="E23" t="s">
+        <v>32</v>
+      </c>
+      <c r="F23" t="s">
+        <v>34</v>
+      </c>
+      <c r="G23" s="5">
+        <v>6.1</v>
+      </c>
+      <c r="H23" s="5">
+        <v>10.029999999999999</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A24" t="s">
         <v>23</v>
       </c>
-      <c r="B24">
+      <c r="B24" s="1">
         <v>30</v>
       </c>
-      <c r="C24">
+      <c r="C24" s="1">
         <v>30.5</v>
       </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="D24" t="s">
+        <v>28</v>
+      </c>
+      <c r="E24" t="s">
+        <v>32</v>
+      </c>
+      <c r="F24" t="s">
+        <v>34</v>
+      </c>
+      <c r="G24" s="5">
+        <v>6.1</v>
+      </c>
+      <c r="H24" s="5">
+        <v>10.029999999999999</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" t="s">
         <v>24</v>
       </c>
-      <c r="B25">
+      <c r="B25" s="1">
         <v>2</v>
       </c>
-      <c r="C25">
+      <c r="C25" s="1">
         <v>2</v>
       </c>
+      <c r="D25" t="s">
+        <v>28</v>
+      </c>
+      <c r="E25" t="s">
+        <v>32</v>
+      </c>
+      <c r="F25" t="s">
+        <v>34</v>
+      </c>
+      <c r="G25" s="5">
+        <v>6.1</v>
+      </c>
+      <c r="H25" s="5">
+        <v>10.029999999999999</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="G26" s="5"/>
+      <c r="H26" s="5"/>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="G27" s="5"/>
+      <c r="H27" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>